<commit_message>
chore: update Taipower natural gas prices
</commit_message>
<xml_diff>
--- a/output/taipower_natural_gas_prices_all.xlsx
+++ b/output/taipower_natural_gas_prices_all.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,6 +501,47 @@
       <c r="I2" t="inlineStr">
         <is>
           <t>7b9dc0b060b2bd777361314762e7ca9f99d1d9e0d8f0a4ca2b578794a37d8e76</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-25T05:46:14.313592+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://www.taipower.com.tw/2289/2363/2373/2377/10367/normalPost</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>台灣中油115年4月發電用戶天然氣牌價</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>17.8485</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>115年1-4月</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>5083</v>
+      </c>
+      <c r="H3" t="n">
+        <v>13.7618</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>61ad93d613af4cd667f369a9de0fa8eb62e9bebd5949e226ddb13ccfffc36682</t>
         </is>
       </c>
     </row>

</xml_diff>